<commit_message>
Fix : token storage
</commit_message>
<xml_diff>
--- a/backend/expense_details.xlsx
+++ b/backend/expense_details.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,91 +415,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>sdfhsfdh</v>
+        <v>ffb</v>
       </c>
       <c r="B2">
-        <v>346457</v>
+        <v>435</v>
       </c>
       <c r="C2" t="str">
         <v>Food</v>
       </c>
       <c r="D2" t="str">
-        <v>5/5/2026</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>335</v>
-      </c>
-      <c r="B3">
-        <v>345</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Food</v>
-      </c>
-      <c r="D3" t="str">
-        <v>5/5/2026</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>fghg</v>
-      </c>
-      <c r="B4">
-        <v>34667</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Investments</v>
-      </c>
-      <c r="D4" t="str">
-        <v>5/5/2026</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>fhv</v>
-      </c>
-      <c r="B5">
-        <v>7587</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Food</v>
-      </c>
-      <c r="D5" t="str">
-        <v>5/5/2026</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>fhv</v>
-      </c>
-      <c r="B6">
-        <v>7587</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Food</v>
-      </c>
-      <c r="D6" t="str">
-        <v>5/5/2026</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>sdf</v>
-      </c>
-      <c r="B7">
-        <v>325</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Housing</v>
-      </c>
-      <c r="D7" t="str">
-        <v>5/5/2026</v>
+        <v>8/5/2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>